<commit_message>
adding screenshot based eval and enabling pass@k evaluation
</commit_message>
<xml_diff>
--- a/research/results/171225/summary_eval.xlsx
+++ b/research/results/171225/summary_eval.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Summary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3287,4 +3288,960 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>query_index</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>query</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>data_file</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>hierarchical_column_header__diversified</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>merge_similar_columns__diversified</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>single_hierarchical_row_header__diversified</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>transpose_table__diversified</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>hierarchical_column_header__disturbed</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>merge_similar_columns__disturbed</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>single_hierarchical_row_header__disturbed</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>transpose_table__disturbed</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Retail_Sales_Orders_original_0</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Looking at all the sales orders, what is the total revenue (NetAmount) generated in each region, and can you list them in descending order of revenue?</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>dev_test/Diversification/Self Created Dataset/Manual Created Dataset/Normal Diversifications/Retail_Sales_Orders/Retail_Sales_Orders_original.xlsx</t>
+        </is>
+      </c>
+      <c r="D2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J2" t="b">
+        <v>1</v>
+      </c>
+      <c r="K2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Retail_Sales_Orders_original_1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Which product sold the most units overall across all orders? (mention only the product name)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>dev_test/Diversification/Self Created Dataset/Manual Created Dataset/Normal Diversifications/Retail_Sales_Orders/Retail_Sales_Orders_original.xlsx</t>
+        </is>
+      </c>
+      <c r="D3" t="b">
+        <v>1</v>
+      </c>
+      <c r="E3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I3" t="b">
+        <v>1</v>
+      </c>
+      <c r="J3" t="b">
+        <v>1</v>
+      </c>
+      <c r="K3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Retail_Sales_Orders_original_2</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>What is the average discount rate (rounded to 3 decimals) applied to orders shipped via Express compared to those shipped via Standard?</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>dev_test/Diversification/Self Created Dataset/Manual Created Dataset/Normal Diversifications/Retail_Sales_Orders/Retail_Sales_Orders_original.xlsx</t>
+        </is>
+      </c>
+      <c r="D4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" t="b">
+        <v>0</v>
+      </c>
+      <c r="H4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J4" t="b">
+        <v>1</v>
+      </c>
+      <c r="K4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Retail_Sales_Orders_original_3</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>What percentage of orders were delivered within two days of the order date?</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>dev_test/Diversification/Self Created Dataset/Manual Created Dataset/Normal Diversifications/Retail_Sales_Orders/Retail_Sales_Orders_original.xlsx</t>
+        </is>
+      </c>
+      <c r="D5" t="b">
+        <v>1</v>
+      </c>
+      <c r="E5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I5" t="b">
+        <v>1</v>
+      </c>
+      <c r="J5" t="b">
+        <v>1</v>
+      </c>
+      <c r="K5" t="b">
+        <v>1</v>
+      </c>
+      <c r="L5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>HR_Timesheets_original_0</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>For all billable entries, what is the total revenue generated grouped by project?</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>dev_test/Diversification/Self Created Dataset/Manual Created Dataset/Normal Diversifications/HR_Timesheets/HR_Timesheets_original.xlsx</t>
+        </is>
+      </c>
+      <c r="D6" t="b">
+        <v>1</v>
+      </c>
+      <c r="E6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" t="b">
+        <v>1</v>
+      </c>
+      <c r="G6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H6" t="b">
+        <v>1</v>
+      </c>
+      <c r="I6" t="b">
+        <v>1</v>
+      </c>
+      <c r="J6" t="b">
+        <v>1</v>
+      </c>
+      <c r="K6" t="b">
+        <v>0</v>
+      </c>
+      <c r="L6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>HR_Timesheets_original_1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>How many employees did overtime?</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>dev_test/Diversification/Self Created Dataset/Manual Created Dataset/Normal Diversifications/HR_Timesheets/HR_Timesheets_original.xlsx</t>
+        </is>
+      </c>
+      <c r="D7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E7" t="b">
+        <v>0</v>
+      </c>
+      <c r="F7" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" t="b">
+        <v>1</v>
+      </c>
+      <c r="I7" t="b">
+        <v>1</v>
+      </c>
+      <c r="J7" t="b">
+        <v>1</v>
+      </c>
+      <c r="K7" t="b">
+        <v>1</v>
+      </c>
+      <c r="L7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>HR_Timesheets_original_2</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>What is the average number of hours worked for employees working remotely compared to those onsite?</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>dev_test/Diversification/Self Created Dataset/Manual Created Dataset/Normal Diversifications/HR_Timesheets/HR_Timesheets_original.xlsx</t>
+        </is>
+      </c>
+      <c r="D8" t="b">
+        <v>1</v>
+      </c>
+      <c r="E8" t="b">
+        <v>1</v>
+      </c>
+      <c r="F8" t="b">
+        <v>1</v>
+      </c>
+      <c r="G8" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" t="b">
+        <v>1</v>
+      </c>
+      <c r="I8" t="b">
+        <v>1</v>
+      </c>
+      <c r="J8" t="b">
+        <v>1</v>
+      </c>
+      <c r="K8" t="b">
+        <v>1</v>
+      </c>
+      <c r="L8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Logistics_Shipments_original_0</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>What is the average number of transit days for each carrier for Standard priority level?</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>dev_test/Diversification/Self Created Dataset/Manual Created Dataset/Normal Diversifications/Logistics_Shipments/Logistics_Shipments_original.xlsx</t>
+        </is>
+      </c>
+      <c r="D9" t="b">
+        <v>1</v>
+      </c>
+      <c r="E9" t="b">
+        <v>1</v>
+      </c>
+      <c r="F9" t="b">
+        <v>1</v>
+      </c>
+      <c r="G9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" t="b">
+        <v>1</v>
+      </c>
+      <c r="I9" t="b">
+        <v>1</v>
+      </c>
+      <c r="J9" t="b">
+        <v>1</v>
+      </c>
+      <c r="K9" t="b">
+        <v>1</v>
+      </c>
+      <c r="L9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Logistics_Shipments_original_1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Which three destinations received the highest total shipment weight?</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>dev_test/Diversification/Self Created Dataset/Manual Created Dataset/Normal Diversifications/Logistics_Shipments/Logistics_Shipments_original.xlsx</t>
+        </is>
+      </c>
+      <c r="D10" t="b">
+        <v>1</v>
+      </c>
+      <c r="E10" t="b">
+        <v>1</v>
+      </c>
+      <c r="F10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K10" t="b">
+        <v>1</v>
+      </c>
+      <c r="L10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Logistics_Shipments_original_2</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>What percentage of shipments met the on-time delivery rule (Priority ≤ 4 days, Standard ≤ 6 days), rounded to nearest integer?</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>dev_test/Diversification/Self Created Dataset/Manual Created Dataset/Normal Diversifications/Logistics_Shipments/Logistics_Shipments_original.xlsx</t>
+        </is>
+      </c>
+      <c r="D11" t="b">
+        <v>1</v>
+      </c>
+      <c r="E11" t="b">
+        <v>1</v>
+      </c>
+      <c r="F11" t="b">
+        <v>1</v>
+      </c>
+      <c r="G11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I11" t="b">
+        <v>1</v>
+      </c>
+      <c r="J11" t="b">
+        <v>1</v>
+      </c>
+      <c r="K11" t="b">
+        <v>1</v>
+      </c>
+      <c r="L11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Clinic_Visits_original_0</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>What is the median systolic blood pressure recorded for patients grouped by their medical condition?</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>dev_test/Diversification/Self Created Dataset/Manual Created Dataset/Normal Diversifications/Clinic_Visits/Clinic_Visits_original.xlsx</t>
+        </is>
+      </c>
+      <c r="D12" t="b">
+        <v>1</v>
+      </c>
+      <c r="E12" t="b">
+        <v>1</v>
+      </c>
+      <c r="F12" t="b">
+        <v>1</v>
+      </c>
+      <c r="G12" t="b">
+        <v>1</v>
+      </c>
+      <c r="H12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I12" t="b">
+        <v>1</v>
+      </c>
+      <c r="J12" t="b">
+        <v>1</v>
+      </c>
+      <c r="K12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Clinic_Visits_original_1</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>For each doctor, what proportion of their visits required a follow-up?</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>dev_test/Diversification/Self Created Dataset/Manual Created Dataset/Normal Diversifications/Clinic_Visits/Clinic_Visits_original.xlsx</t>
+        </is>
+      </c>
+      <c r="D13" t="b">
+        <v>1</v>
+      </c>
+      <c r="E13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F13" t="b">
+        <v>1</v>
+      </c>
+      <c r="G13" t="b">
+        <v>1</v>
+      </c>
+      <c r="H13" t="b">
+        <v>1</v>
+      </c>
+      <c r="I13" t="b">
+        <v>1</v>
+      </c>
+      <c r="J13" t="b">
+        <v>1</v>
+      </c>
+      <c r="K13" t="b">
+        <v>1</v>
+      </c>
+      <c r="L13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Clinic_Visits_original_2</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>What is the average consultation fee for females grouped by condition?</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>dev_test/Diversification/Self Created Dataset/Manual Created Dataset/Normal Diversifications/Clinic_Visits/Clinic_Visits_original.xlsx</t>
+        </is>
+      </c>
+      <c r="D14" t="b">
+        <v>1</v>
+      </c>
+      <c r="E14" t="b">
+        <v>1</v>
+      </c>
+      <c r="F14" t="b">
+        <v>1</v>
+      </c>
+      <c r="G14" t="b">
+        <v>0</v>
+      </c>
+      <c r="H14" t="b">
+        <v>1</v>
+      </c>
+      <c r="I14" t="b">
+        <v>1</v>
+      </c>
+      <c r="J14" t="b">
+        <v>1</v>
+      </c>
+      <c r="K14" t="b">
+        <v>0</v>
+      </c>
+      <c r="L14" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Personal_Finance_Transactions_original_0</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>What is the total spending for each category in the month of June?</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>dev_test/Diversification/Self Created Dataset/Manual Created Dataset/Normal Diversifications/Personal_Finance_Transactions/Personal_Finance_Transactions_original.xlsx</t>
+        </is>
+      </c>
+      <c r="D15" t="b">
+        <v>1</v>
+      </c>
+      <c r="E15" t="b">
+        <v>1</v>
+      </c>
+      <c r="F15" t="b">
+        <v>1</v>
+      </c>
+      <c r="G15" t="b">
+        <v>0</v>
+      </c>
+      <c r="H15" t="b">
+        <v>0</v>
+      </c>
+      <c r="I15" t="b">
+        <v>1</v>
+      </c>
+      <c r="J15" t="b">
+        <v>1</v>
+      </c>
+      <c r="K15" t="b">
+        <v>0</v>
+      </c>
+      <c r="L15" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Personal_Finance_Transactions_original_1</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Which payment method (mention only name) earned the highest total cashback?</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>dev_test/Diversification/Self Created Dataset/Manual Created Dataset/Normal Diversifications/Personal_Finance_Transactions/Personal_Finance_Transactions_original.xlsx</t>
+        </is>
+      </c>
+      <c r="D16" t="b">
+        <v>1</v>
+      </c>
+      <c r="E16" t="b">
+        <v>1</v>
+      </c>
+      <c r="F16" t="b">
+        <v>1</v>
+      </c>
+      <c r="G16" t="b">
+        <v>1</v>
+      </c>
+      <c r="H16" t="b">
+        <v>1</v>
+      </c>
+      <c r="I16" t="b">
+        <v>1</v>
+      </c>
+      <c r="J16" t="b">
+        <v>1</v>
+      </c>
+      <c r="K16" t="b">
+        <v>1</v>
+      </c>
+      <c r="L16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Personal_Finance_Transactions_original_2</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>What percent of total spending was on recurring expenses?</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>dev_test/Diversification/Self Created Dataset/Manual Created Dataset/Normal Diversifications/Personal_Finance_Transactions/Personal_Finance_Transactions_original.xlsx</t>
+        </is>
+      </c>
+      <c r="D17" t="b">
+        <v>1</v>
+      </c>
+      <c r="E17" t="b">
+        <v>1</v>
+      </c>
+      <c r="F17" t="b">
+        <v>1</v>
+      </c>
+      <c r="G17" t="b">
+        <v>0</v>
+      </c>
+      <c r="H17" t="b">
+        <v>1</v>
+      </c>
+      <c r="I17" t="b">
+        <v>1</v>
+      </c>
+      <c r="J17" t="b">
+        <v>1</v>
+      </c>
+      <c r="K17" t="b">
+        <v>0</v>
+      </c>
+      <c r="L17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>University_Grades_original_0</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>What is the average total score for each course with a 100% pass rate?</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>dev_test/Diversification/Self Created Dataset/Manual Created Dataset/Normal Diversifications/University_Grades/University_Grades_original.xlsx</t>
+        </is>
+      </c>
+      <c r="D18" t="b">
+        <v>1</v>
+      </c>
+      <c r="E18" t="b">
+        <v>1</v>
+      </c>
+      <c r="F18" t="b">
+        <v>1</v>
+      </c>
+      <c r="G18" t="b">
+        <v>1</v>
+      </c>
+      <c r="H18" t="b">
+        <v>0</v>
+      </c>
+      <c r="I18" t="b">
+        <v>1</v>
+      </c>
+      <c r="J18" t="b">
+        <v>1</v>
+      </c>
+      <c r="K18" t="b">
+        <v>1</v>
+      </c>
+      <c r="L18" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>University_Grades_original_1</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>How many students received grade A?</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>dev_test/Diversification/Self Created Dataset/Manual Created Dataset/Normal Diversifications/University_Grades/University_Grades_original.xlsx</t>
+        </is>
+      </c>
+      <c r="D19" t="b">
+        <v>1</v>
+      </c>
+      <c r="E19" t="b">
+        <v>1</v>
+      </c>
+      <c r="F19" t="b">
+        <v>1</v>
+      </c>
+      <c r="G19" t="b">
+        <v>1</v>
+      </c>
+      <c r="H19" t="b">
+        <v>1</v>
+      </c>
+      <c r="I19" t="b">
+        <v>1</v>
+      </c>
+      <c r="J19" t="b">
+        <v>1</v>
+      </c>
+      <c r="K19" t="b">
+        <v>1</v>
+      </c>
+      <c r="L19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>University_Grades_original_2</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Which professor (only name) achieved the highest average project score?</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>dev_test/Diversification/Self Created Dataset/Manual Created Dataset/Normal Diversifications/University_Grades/University_Grades_original.xlsx</t>
+        </is>
+      </c>
+      <c r="D20" t="b">
+        <v>1</v>
+      </c>
+      <c r="E20" t="b">
+        <v>1</v>
+      </c>
+      <c r="F20" t="b">
+        <v>0</v>
+      </c>
+      <c r="G20" t="b">
+        <v>1</v>
+      </c>
+      <c r="H20" t="b">
+        <v>1</v>
+      </c>
+      <c r="I20" t="b">
+        <v>1</v>
+      </c>
+      <c r="J20" t="b">
+        <v>1</v>
+      </c>
+      <c r="K20" t="b">
+        <v>1</v>
+      </c>
+      <c r="L20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>University_Grades_original_3</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Among all students, which student achieved the highest overall score, and what was their total marks along with the corresponding letter grade? Mention as a dictionary with keys 'StudentID', 'Marks', and 'Grade'.</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>dev_test/Diversification/Self Created Dataset/Manual Created Dataset/Normal Diversifications/University_Grades/University_Grades_original.xlsx</t>
+        </is>
+      </c>
+      <c r="D21" t="b">
+        <v>1</v>
+      </c>
+      <c r="E21" t="b">
+        <v>1</v>
+      </c>
+      <c r="F21" t="b">
+        <v>1</v>
+      </c>
+      <c r="G21" t="b">
+        <v>1</v>
+      </c>
+      <c r="H21" t="b">
+        <v>1</v>
+      </c>
+      <c r="I21" t="b">
+        <v>1</v>
+      </c>
+      <c r="J21" t="b">
+        <v>1</v>
+      </c>
+      <c r="K21" t="b">
+        <v>1</v>
+      </c>
+      <c r="L21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>